<commit_message>
Corrida | SFE-RMP | 2026-06-24 09:52:40.391115
</commit_message>
<xml_diff>
--- a/indicadores/SFE-RMP_out.xlsx
+++ b/indicadores/SFE-RMP_out.xlsx
@@ -113,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">17/06/2026</t>
+    <t xml:space="preserve">24/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">focampo</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2146,9 +2146,7 @@
       <c r="J7" s="1"/>
     </row>
     <row r="8">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
+      <c r="A8"/>
       <c r="B8"/>
       <c r="C8"/>
       <c r="D8"/>
@@ -2160,14 +2158,10 @@
       <c r="J8" s="1"/>
     </row>
     <row r="9">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
+      <c r="A9"/>
       <c r="B9"/>
       <c r="C9"/>
-      <c r="D9" t="n">
-        <v>0.483805246125811</v>
-      </c>
+      <c r="D9"/>
       <c r="E9"/>
       <c r="F9"/>
       <c r="G9"/>
@@ -2177,13 +2171,11 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
+      <c r="D10"/>
       <c r="E10"/>
       <c r="F10"/>
       <c r="G10"/>
@@ -2192,10 +2184,14 @@
       <c r="J10" s="1"/>
     </row>
     <row r="11">
-      <c r="A11"/>
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
       <c r="B11"/>
       <c r="C11"/>
-      <c r="D11"/>
+      <c r="D11" t="n">
+        <v>0.488435930066107</v>
+      </c>
       <c r="E11"/>
       <c r="F11"/>
       <c r="G11"/>
@@ -2205,11 +2201,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
-      <c r="D12"/>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
       <c r="E12"/>
       <c r="F12"/>
       <c r="G12"/>
@@ -2218,14 +2216,10 @@
       <c r="J12" s="1"/>
     </row>
     <row r="13">
-      <c r="A13" t="s">
-        <v>25</v>
-      </c>
+      <c r="A13"/>
       <c r="B13"/>
       <c r="C13"/>
-      <c r="D13" t="n">
-        <v>0.234067516178856</v>
-      </c>
+      <c r="D13"/>
       <c r="E13"/>
       <c r="F13"/>
       <c r="G13"/>
@@ -2234,7 +2228,9 @@
       <c r="J13" s="1"/>
     </row>
     <row r="14">
-      <c r="A14"/>
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
       <c r="B14"/>
       <c r="C14"/>
       <c r="D14"/>
@@ -2247,11 +2243,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
-      <c r="D15"/>
+      <c r="D15" t="n">
+        <v>0.238569657779543</v>
+      </c>
       <c r="E15"/>
       <c r="F15"/>
       <c r="G15"/>
@@ -2260,9 +2258,7 @@
       <c r="J15" s="1"/>
     </row>
     <row r="16">
-      <c r="A16" t="s">
-        <v>27</v>
-      </c>
+      <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
@@ -2275,7 +2271,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2289,13 +2285,11 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
-      <c r="D18" t="n">
-        <v>0.000362514669975845</v>
-      </c>
+      <c r="D18"/>
       <c r="E18"/>
       <c r="F18"/>
       <c r="G18"/>
@@ -2305,7 +2299,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2324,7 +2318,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000001899738812327</v>
+        <v>0.000386004168957425</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2334,7 +2328,9 @@
       <c r="J20" s="1"/>
     </row>
     <row r="21">
-      <c r="A21"/>
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
       <c r="B21"/>
       <c r="C21"/>
       <c r="D21"/>
@@ -2346,10 +2342,14 @@
       <c r="J21" s="1"/>
     </row>
     <row r="22">
-      <c r="A22"/>
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
       <c r="B22"/>
       <c r="C22"/>
-      <c r="D22"/>
+      <c r="D22" t="n">
+        <v>0.00000193552741763611</v>
+      </c>
       <c r="E22"/>
       <c r="F22"/>
       <c r="G22"/>
@@ -26841,7 +26841,7 @@
         <v>519</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.070317893467376</v>
+        <v>-0.0680075934442373</v>
       </c>
     </row>
     <row r="6">
@@ -26849,7 +26849,7 @@
         <v>520</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0256826169008705</v>
+        <v>-0.0294829030659208</v>
       </c>
     </row>
     <row r="7">
@@ -26857,7 +26857,7 @@
         <v>521</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0201385499812574</v>
+        <v>0.0092006794638114</v>
       </c>
     </row>
     <row r="8">
@@ -26865,7 +26865,7 @@
         <v>522</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0730115604418791</v>
+        <v>0.0562635272719007</v>
       </c>
     </row>
     <row r="9">
@@ -26873,7 +26873,7 @@
         <v>523</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.131316387930399</v>
+        <v>0.115025340838716</v>
       </c>
     </row>
     <row r="10">
@@ -26881,7 +26881,7 @@
         <v>524</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.209109127005448</v>
+        <v>0.199831022345146</v>
       </c>
     </row>
     <row r="11">
@@ -26889,7 +26889,7 @@
         <v>525</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.296733931781201</v>
+        <v>0.289139893869599</v>
       </c>
     </row>
     <row r="12">
@@ -26897,7 +26897,7 @@
         <v>526</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.398248067508553</v>
+        <v>0.386906199257398</v>
       </c>
     </row>
     <row r="13">
@@ -26905,7 +26905,7 @@
         <v>527</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.477830640682718</v>
+        <v>0.473049718169451</v>
       </c>
     </row>
     <row r="14">
@@ -26913,7 +26913,7 @@
         <v>528</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.483805246125811</v>
+        <v>0.488435930066107</v>
       </c>
     </row>
     <row r="15">
@@ -26921,7 +26921,7 @@
         <v>529</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.45645729934514</v>
+        <v>0.458136073122225</v>
       </c>
     </row>
     <row r="16">
@@ -26929,7 +26929,7 @@
         <v>530</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.438190692287671</v>
+        <v>0.435098877540727</v>
       </c>
     </row>
     <row r="17">
@@ -26937,7 +26937,7 @@
         <v>531</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.41343377727187</v>
+        <v>0.41092472054468</v>
       </c>
     </row>
     <row r="18">
@@ -26945,7 +26945,7 @@
         <v>532</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.393738882465807</v>
+        <v>0.389960906243912</v>
       </c>
     </row>
     <row r="19">
@@ -26953,7 +26953,7 @@
         <v>533</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.394530072473975</v>
+        <v>0.388238450178117</v>
       </c>
     </row>
     <row r="20">
@@ -26961,7 +26961,7 @@
         <v>534</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.395056631458851</v>
+        <v>0.390950115543832</v>
       </c>
     </row>
     <row r="21">
@@ -26969,7 +26969,7 @@
         <v>535</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.380569675710534</v>
+        <v>0.381972115014119</v>
       </c>
     </row>
     <row r="22">
@@ -26977,7 +26977,7 @@
         <v>536</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.345525586033416</v>
+        <v>0.346342650040605</v>
       </c>
     </row>
     <row r="23">
@@ -26985,7 +26985,7 @@
         <v>537</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.3111517292173</v>
+        <v>0.306382774471776</v>
       </c>
     </row>
     <row r="24">

</xml_diff>